<commit_message>
Added explanation of IN/OUT syntax to Key tab
</commit_message>
<xml_diff>
--- a/CPU Design/CPU opcodes.xlsx
+++ b/CPU Design/CPU opcodes.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4507"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="103" windowWidth="14803" windowHeight="8014" activeTab="1"/>
+    <workbookView xWindow="240" yWindow="103" windowWidth="14803" windowHeight="8014"/>
   </bookViews>
   <sheets>
     <sheet name="opcodes" sheetId="1" r:id="rId1"/>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="147">
   <si>
     <t>Mnemonic</t>
   </si>
@@ -655,6 +655,52 @@
         <scheme val="minor"/>
       </rPr>
       <t>Address</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Port[Ra]=Rb </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>means write value in Rb to output port number specified by Ra</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Rb=Port[Ra]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> means Rb = value of input port number specified Ra</t>
     </r>
   </si>
 </sst>
@@ -909,6 +955,52 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="180"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -936,52 +1028,6 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1280,7 +1326,7 @@
   <sheetFormatPr defaultRowHeight="14.6"/>
   <cols>
     <col min="1" max="1" width="16.4609375" customWidth="1"/>
-    <col min="2" max="2" width="33.15234375" style="60" customWidth="1"/>
+    <col min="2" max="2" width="33.15234375" style="36" customWidth="1"/>
     <col min="3" max="3" width="7.4609375" style="1" customWidth="1"/>
     <col min="4" max="4" width="2.07421875" customWidth="1"/>
     <col min="5" max="20" width="2.23046875" style="1" customWidth="1"/>
@@ -1382,28 +1428,28 @@
     </row>
     <row r="3" spans="1:25">
       <c r="A3" s="33"/>
-      <c r="E3" s="36" t="s">
-        <v>1</v>
-      </c>
-      <c r="F3" s="37"/>
-      <c r="G3" s="37"/>
-      <c r="H3" s="37"/>
-      <c r="I3" s="38"/>
+      <c r="E3" s="52" t="s">
+        <v>1</v>
+      </c>
+      <c r="F3" s="53"/>
+      <c r="G3" s="53"/>
+      <c r="H3" s="53"/>
+      <c r="I3" s="54"/>
       <c r="J3" s="7"/>
-      <c r="K3" s="39" t="s">
+      <c r="K3" s="55" t="s">
         <v>30</v>
       </c>
-      <c r="L3" s="40"/>
-      <c r="M3" s="40"/>
-      <c r="N3" s="40"/>
-      <c r="O3" s="41"/>
-      <c r="P3" s="42" t="s">
+      <c r="L3" s="56"/>
+      <c r="M3" s="56"/>
+      <c r="N3" s="56"/>
+      <c r="O3" s="57"/>
+      <c r="P3" s="58" t="s">
         <v>31</v>
       </c>
-      <c r="Q3" s="43"/>
-      <c r="R3" s="43"/>
-      <c r="S3" s="43"/>
-      <c r="T3" s="44"/>
+      <c r="Q3" s="59"/>
+      <c r="R3" s="59"/>
+      <c r="S3" s="59"/>
+      <c r="T3" s="60"/>
     </row>
     <row r="4" spans="1:25">
       <c r="A4" s="33"/>
@@ -1448,7 +1494,7 @@
       <c r="A5" s="33" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="60" t="s">
+      <c r="B5" s="36" t="s">
         <v>78</v>
       </c>
       <c r="C5" s="1">
@@ -2208,30 +2254,30 @@
     <row r="17" spans="1:25">
       <c r="A17" s="33"/>
       <c r="C17"/>
-      <c r="E17" s="45" t="s">
-        <v>1</v>
-      </c>
-      <c r="F17" s="46"/>
-      <c r="G17" s="46"/>
-      <c r="H17" s="46"/>
-      <c r="I17" s="47"/>
-      <c r="J17" s="48" t="s">
+      <c r="E17" s="37" t="s">
+        <v>1</v>
+      </c>
+      <c r="F17" s="38"/>
+      <c r="G17" s="38"/>
+      <c r="H17" s="38"/>
+      <c r="I17" s="39"/>
+      <c r="J17" s="40" t="s">
         <v>47</v>
       </c>
-      <c r="K17" s="49"/>
-      <c r="L17" s="50"/>
-      <c r="M17" s="51" t="s">
+      <c r="K17" s="41"/>
+      <c r="L17" s="42"/>
+      <c r="M17" s="43" t="s">
         <v>48</v>
       </c>
-      <c r="N17" s="52"/>
-      <c r="O17" s="52"/>
-      <c r="P17" s="53"/>
-      <c r="Q17" s="54" t="s">
+      <c r="N17" s="44"/>
+      <c r="O17" s="44"/>
+      <c r="P17" s="45"/>
+      <c r="Q17" s="46" t="s">
         <v>49</v>
       </c>
-      <c r="R17" s="55"/>
-      <c r="S17" s="55"/>
-      <c r="T17" s="56"/>
+      <c r="R17" s="47"/>
+      <c r="S17" s="47"/>
+      <c r="T17" s="48"/>
     </row>
     <row r="18" spans="1:25">
       <c r="A18" s="33" t="s">
@@ -2568,28 +2614,28 @@
     </row>
     <row r="24" spans="1:25">
       <c r="A24" s="33"/>
-      <c r="E24" s="45" t="s">
-        <v>1</v>
-      </c>
-      <c r="F24" s="46"/>
-      <c r="G24" s="46"/>
-      <c r="H24" s="46"/>
-      <c r="I24" s="47"/>
-      <c r="J24" s="48" t="s">
+      <c r="E24" s="37" t="s">
+        <v>1</v>
+      </c>
+      <c r="F24" s="38"/>
+      <c r="G24" s="38"/>
+      <c r="H24" s="38"/>
+      <c r="I24" s="39"/>
+      <c r="J24" s="40" t="s">
         <v>47</v>
       </c>
-      <c r="K24" s="49"/>
-      <c r="L24" s="50"/>
-      <c r="M24" s="51" t="s">
+      <c r="K24" s="41"/>
+      <c r="L24" s="42"/>
+      <c r="M24" s="43" t="s">
         <v>48</v>
       </c>
-      <c r="N24" s="52"/>
-      <c r="O24" s="52"/>
-      <c r="P24" s="53"/>
-      <c r="Q24" s="57"/>
-      <c r="R24" s="58"/>
-      <c r="S24" s="58"/>
-      <c r="T24" s="59"/>
+      <c r="N24" s="44"/>
+      <c r="O24" s="44"/>
+      <c r="P24" s="45"/>
+      <c r="Q24" s="49"/>
+      <c r="R24" s="50"/>
+      <c r="S24" s="50"/>
+      <c r="T24" s="51"/>
     </row>
     <row r="25" spans="1:25">
       <c r="A25" s="33" t="s">
@@ -2663,28 +2709,28 @@
     <row r="27" spans="1:25">
       <c r="A27" s="33"/>
       <c r="C27"/>
-      <c r="E27" s="45" t="s">
-        <v>1</v>
-      </c>
-      <c r="F27" s="46"/>
-      <c r="G27" s="46"/>
-      <c r="H27" s="46"/>
-      <c r="I27" s="47"/>
-      <c r="J27" s="57"/>
-      <c r="K27" s="58"/>
-      <c r="L27" s="59"/>
-      <c r="M27" s="51" t="s">
+      <c r="E27" s="37" t="s">
+        <v>1</v>
+      </c>
+      <c r="F27" s="38"/>
+      <c r="G27" s="38"/>
+      <c r="H27" s="38"/>
+      <c r="I27" s="39"/>
+      <c r="J27" s="49"/>
+      <c r="K27" s="50"/>
+      <c r="L27" s="51"/>
+      <c r="M27" s="43" t="s">
         <v>48</v>
       </c>
-      <c r="N27" s="52"/>
-      <c r="O27" s="52"/>
-      <c r="P27" s="53"/>
-      <c r="Q27" s="54" t="s">
+      <c r="N27" s="44"/>
+      <c r="O27" s="44"/>
+      <c r="P27" s="45"/>
+      <c r="Q27" s="46" t="s">
         <v>49</v>
       </c>
-      <c r="R27" s="55"/>
-      <c r="S27" s="55"/>
-      <c r="T27" s="56"/>
+      <c r="R27" s="47"/>
+      <c r="S27" s="47"/>
+      <c r="T27" s="48"/>
     </row>
     <row r="28" spans="1:25">
       <c r="A28" s="33" t="s">
@@ -2757,26 +2803,26 @@
     </row>
     <row r="30" spans="1:25">
       <c r="A30" s="33"/>
-      <c r="E30" s="45" t="s">
-        <v>1</v>
-      </c>
-      <c r="F30" s="46"/>
-      <c r="G30" s="46"/>
-      <c r="H30" s="46"/>
-      <c r="I30" s="47"/>
-      <c r="J30" s="57"/>
-      <c r="K30" s="58"/>
-      <c r="L30" s="59"/>
-      <c r="M30" s="51" t="s">
+      <c r="E30" s="37" t="s">
+        <v>1</v>
+      </c>
+      <c r="F30" s="38"/>
+      <c r="G30" s="38"/>
+      <c r="H30" s="38"/>
+      <c r="I30" s="39"/>
+      <c r="J30" s="49"/>
+      <c r="K30" s="50"/>
+      <c r="L30" s="51"/>
+      <c r="M30" s="43" t="s">
         <v>48</v>
       </c>
-      <c r="N30" s="52"/>
-      <c r="O30" s="52"/>
-      <c r="P30" s="53"/>
-      <c r="Q30" s="57"/>
-      <c r="R30" s="58"/>
-      <c r="S30" s="58"/>
-      <c r="T30" s="59"/>
+      <c r="N30" s="44"/>
+      <c r="O30" s="44"/>
+      <c r="P30" s="45"/>
+      <c r="Q30" s="49"/>
+      <c r="R30" s="50"/>
+      <c r="S30" s="50"/>
+      <c r="T30" s="51"/>
     </row>
     <row r="31" spans="1:25">
       <c r="A31" s="33" t="s">
@@ -2849,28 +2895,28 @@
     </row>
     <row r="33" spans="1:25">
       <c r="A33" s="33"/>
-      <c r="E33" s="45" t="s">
-        <v>1</v>
-      </c>
-      <c r="F33" s="46"/>
-      <c r="G33" s="46"/>
-      <c r="H33" s="46"/>
-      <c r="I33" s="47"/>
-      <c r="J33" s="48" t="s">
+      <c r="E33" s="37" t="s">
+        <v>1</v>
+      </c>
+      <c r="F33" s="38"/>
+      <c r="G33" s="38"/>
+      <c r="H33" s="38"/>
+      <c r="I33" s="39"/>
+      <c r="J33" s="40" t="s">
         <v>47</v>
       </c>
-      <c r="K33" s="49"/>
-      <c r="L33" s="50"/>
-      <c r="M33" s="51" t="s">
+      <c r="K33" s="41"/>
+      <c r="L33" s="42"/>
+      <c r="M33" s="43" t="s">
         <v>48</v>
       </c>
-      <c r="N33" s="52"/>
-      <c r="O33" s="52"/>
-      <c r="P33" s="53"/>
-      <c r="Q33" s="57"/>
-      <c r="R33" s="58"/>
-      <c r="S33" s="58"/>
-      <c r="T33" s="59"/>
+      <c r="N33" s="44"/>
+      <c r="O33" s="44"/>
+      <c r="P33" s="45"/>
+      <c r="Q33" s="49"/>
+      <c r="R33" s="50"/>
+      <c r="S33" s="50"/>
+      <c r="T33" s="51"/>
     </row>
     <row r="34" spans="1:25">
       <c r="A34" s="33" t="s">
@@ -2943,28 +2989,28 @@
     </row>
     <row r="36" spans="1:25">
       <c r="A36" s="33"/>
-      <c r="E36" s="45" t="s">
-        <v>1</v>
-      </c>
-      <c r="F36" s="46"/>
-      <c r="G36" s="46"/>
-      <c r="H36" s="46"/>
-      <c r="I36" s="47"/>
-      <c r="J36" s="48" t="s">
+      <c r="E36" s="37" t="s">
+        <v>1</v>
+      </c>
+      <c r="F36" s="38"/>
+      <c r="G36" s="38"/>
+      <c r="H36" s="38"/>
+      <c r="I36" s="39"/>
+      <c r="J36" s="40" t="s">
         <v>47</v>
       </c>
-      <c r="K36" s="49"/>
-      <c r="L36" s="50"/>
-      <c r="M36" s="51" t="s">
+      <c r="K36" s="41"/>
+      <c r="L36" s="42"/>
+      <c r="M36" s="43" t="s">
         <v>48</v>
       </c>
-      <c r="N36" s="52"/>
-      <c r="O36" s="52"/>
-      <c r="P36" s="53"/>
-      <c r="Q36" s="57"/>
-      <c r="R36" s="58"/>
-      <c r="S36" s="58"/>
-      <c r="T36" s="59"/>
+      <c r="N36" s="44"/>
+      <c r="O36" s="44"/>
+      <c r="P36" s="45"/>
+      <c r="Q36" s="49"/>
+      <c r="R36" s="50"/>
+      <c r="S36" s="50"/>
+      <c r="T36" s="51"/>
     </row>
     <row r="37" spans="1:25">
       <c r="A37" s="33" t="s">
@@ -3037,30 +3083,30 @@
     </row>
     <row r="39" spans="1:25">
       <c r="A39" s="33"/>
-      <c r="E39" s="45" t="s">
-        <v>1</v>
-      </c>
-      <c r="F39" s="46"/>
-      <c r="G39" s="46"/>
-      <c r="H39" s="46"/>
-      <c r="I39" s="47"/>
-      <c r="J39" s="48" t="s">
+      <c r="E39" s="37" t="s">
+        <v>1</v>
+      </c>
+      <c r="F39" s="38"/>
+      <c r="G39" s="38"/>
+      <c r="H39" s="38"/>
+      <c r="I39" s="39"/>
+      <c r="J39" s="40" t="s">
         <v>47</v>
       </c>
-      <c r="K39" s="49"/>
-      <c r="L39" s="50"/>
-      <c r="M39" s="51" t="s">
+      <c r="K39" s="41"/>
+      <c r="L39" s="42"/>
+      <c r="M39" s="43" t="s">
         <v>48</v>
       </c>
-      <c r="N39" s="52"/>
-      <c r="O39" s="52"/>
-      <c r="P39" s="53"/>
-      <c r="Q39" s="54" t="s">
+      <c r="N39" s="44"/>
+      <c r="O39" s="44"/>
+      <c r="P39" s="45"/>
+      <c r="Q39" s="46" t="s">
         <v>49</v>
       </c>
-      <c r="R39" s="55"/>
-      <c r="S39" s="55"/>
-      <c r="T39" s="56"/>
+      <c r="R39" s="47"/>
+      <c r="S39" s="47"/>
+      <c r="T39" s="48"/>
       <c r="V39" s="3" t="s">
         <v>63</v>
       </c>
@@ -3139,30 +3185,30 @@
     </row>
     <row r="42" spans="1:25">
       <c r="A42" s="33"/>
-      <c r="E42" s="45" t="s">
-        <v>1</v>
-      </c>
-      <c r="F42" s="46"/>
-      <c r="G42" s="46"/>
-      <c r="H42" s="46"/>
-      <c r="I42" s="47"/>
-      <c r="J42" s="48" t="s">
+      <c r="E42" s="37" t="s">
+        <v>1</v>
+      </c>
+      <c r="F42" s="38"/>
+      <c r="G42" s="38"/>
+      <c r="H42" s="38"/>
+      <c r="I42" s="39"/>
+      <c r="J42" s="40" t="s">
         <v>47</v>
       </c>
-      <c r="K42" s="49"/>
-      <c r="L42" s="50"/>
-      <c r="M42" s="51" t="s">
+      <c r="K42" s="41"/>
+      <c r="L42" s="42"/>
+      <c r="M42" s="43" t="s">
         <v>48</v>
       </c>
-      <c r="N42" s="52"/>
-      <c r="O42" s="52"/>
-      <c r="P42" s="53"/>
-      <c r="Q42" s="54" t="s">
+      <c r="N42" s="44"/>
+      <c r="O42" s="44"/>
+      <c r="P42" s="45"/>
+      <c r="Q42" s="46" t="s">
         <v>49</v>
       </c>
-      <c r="R42" s="55"/>
-      <c r="S42" s="55"/>
-      <c r="T42" s="56"/>
+      <c r="R42" s="47"/>
+      <c r="S42" s="47"/>
+      <c r="T42" s="48"/>
       <c r="V42" s="3" t="s">
         <v>66</v>
       </c>
@@ -3241,30 +3287,30 @@
     </row>
     <row r="45" spans="1:25">
       <c r="A45" s="33"/>
-      <c r="E45" s="45" t="s">
-        <v>1</v>
-      </c>
-      <c r="F45" s="46"/>
-      <c r="G45" s="46"/>
-      <c r="H45" s="46"/>
-      <c r="I45" s="47"/>
-      <c r="J45" s="48" t="s">
+      <c r="E45" s="37" t="s">
+        <v>1</v>
+      </c>
+      <c r="F45" s="38"/>
+      <c r="G45" s="38"/>
+      <c r="H45" s="38"/>
+      <c r="I45" s="39"/>
+      <c r="J45" s="40" t="s">
         <v>47</v>
       </c>
-      <c r="K45" s="49"/>
-      <c r="L45" s="50"/>
-      <c r="M45" s="51" t="s">
+      <c r="K45" s="41"/>
+      <c r="L45" s="42"/>
+      <c r="M45" s="43" t="s">
         <v>48</v>
       </c>
-      <c r="N45" s="52"/>
-      <c r="O45" s="52"/>
-      <c r="P45" s="53"/>
-      <c r="Q45" s="54" t="s">
+      <c r="N45" s="44"/>
+      <c r="O45" s="44"/>
+      <c r="P45" s="45"/>
+      <c r="Q45" s="46" t="s">
         <v>49</v>
       </c>
-      <c r="R45" s="55"/>
-      <c r="S45" s="55"/>
-      <c r="T45" s="56"/>
+      <c r="R45" s="47"/>
+      <c r="S45" s="47"/>
+      <c r="T45" s="48"/>
       <c r="V45" s="3" t="s">
         <v>66</v>
       </c>
@@ -3343,28 +3389,28 @@
     </row>
     <row r="48" spans="1:25">
       <c r="A48" s="33"/>
-      <c r="E48" s="45" t="s">
-        <v>1</v>
-      </c>
-      <c r="F48" s="46"/>
-      <c r="G48" s="46"/>
-      <c r="H48" s="46"/>
-      <c r="I48" s="47"/>
-      <c r="J48" s="48" t="s">
+      <c r="E48" s="37" t="s">
+        <v>1</v>
+      </c>
+      <c r="F48" s="38"/>
+      <c r="G48" s="38"/>
+      <c r="H48" s="38"/>
+      <c r="I48" s="39"/>
+      <c r="J48" s="40" t="s">
         <v>47</v>
       </c>
-      <c r="K48" s="49"/>
-      <c r="L48" s="50"/>
-      <c r="M48" s="57"/>
-      <c r="N48" s="58"/>
-      <c r="O48" s="58"/>
-      <c r="P48" s="59"/>
-      <c r="Q48" s="54" t="s">
+      <c r="K48" s="41"/>
+      <c r="L48" s="42"/>
+      <c r="M48" s="49"/>
+      <c r="N48" s="50"/>
+      <c r="O48" s="50"/>
+      <c r="P48" s="51"/>
+      <c r="Q48" s="46" t="s">
         <v>49</v>
       </c>
-      <c r="R48" s="55"/>
-      <c r="S48" s="55"/>
-      <c r="T48" s="56"/>
+      <c r="R48" s="47"/>
+      <c r="S48" s="47"/>
+      <c r="T48" s="48"/>
       <c r="V48" s="3" t="s">
         <v>63</v>
       </c>
@@ -3443,26 +3489,26 @@
     </row>
     <row r="51" spans="1:25">
       <c r="A51" s="33"/>
-      <c r="E51" s="45" t="s">
-        <v>1</v>
-      </c>
-      <c r="F51" s="46"/>
-      <c r="G51" s="46"/>
-      <c r="H51" s="46"/>
-      <c r="I51" s="47"/>
-      <c r="J51" s="57"/>
-      <c r="K51" s="58"/>
-      <c r="L51" s="59"/>
-      <c r="M51" s="51" t="s">
+      <c r="E51" s="37" t="s">
+        <v>1</v>
+      </c>
+      <c r="F51" s="38"/>
+      <c r="G51" s="38"/>
+      <c r="H51" s="38"/>
+      <c r="I51" s="39"/>
+      <c r="J51" s="49"/>
+      <c r="K51" s="50"/>
+      <c r="L51" s="51"/>
+      <c r="M51" s="43" t="s">
         <v>48</v>
       </c>
-      <c r="N51" s="52"/>
-      <c r="O51" s="52"/>
-      <c r="P51" s="53"/>
-      <c r="Q51" s="57"/>
-      <c r="R51" s="58"/>
-      <c r="S51" s="58"/>
-      <c r="T51" s="59"/>
+      <c r="N51" s="44"/>
+      <c r="O51" s="44"/>
+      <c r="P51" s="45"/>
+      <c r="Q51" s="49"/>
+      <c r="R51" s="50"/>
+      <c r="S51" s="50"/>
+      <c r="T51" s="51"/>
     </row>
     <row r="52" spans="1:25">
       <c r="A52" s="33" t="s">
@@ -3535,26 +3581,26 @@
     </row>
     <row r="54" spans="1:25">
       <c r="A54" s="33"/>
-      <c r="E54" s="45" t="s">
-        <v>1</v>
-      </c>
-      <c r="F54" s="46"/>
-      <c r="G54" s="46"/>
-      <c r="H54" s="46"/>
-      <c r="I54" s="47"/>
-      <c r="J54" s="57"/>
-      <c r="K54" s="58"/>
-      <c r="L54" s="59"/>
-      <c r="M54" s="51" t="s">
+      <c r="E54" s="37" t="s">
+        <v>1</v>
+      </c>
+      <c r="F54" s="38"/>
+      <c r="G54" s="38"/>
+      <c r="H54" s="38"/>
+      <c r="I54" s="39"/>
+      <c r="J54" s="49"/>
+      <c r="K54" s="50"/>
+      <c r="L54" s="51"/>
+      <c r="M54" s="43" t="s">
         <v>48</v>
       </c>
-      <c r="N54" s="52"/>
-      <c r="O54" s="52"/>
-      <c r="P54" s="53"/>
-      <c r="Q54" s="57"/>
-      <c r="R54" s="58"/>
-      <c r="S54" s="58"/>
-      <c r="T54" s="59"/>
+      <c r="N54" s="44"/>
+      <c r="O54" s="44"/>
+      <c r="P54" s="45"/>
+      <c r="Q54" s="49"/>
+      <c r="R54" s="50"/>
+      <c r="S54" s="50"/>
+      <c r="T54" s="51"/>
     </row>
     <row r="55" spans="1:25">
       <c r="A55" s="33" t="s">
@@ -3627,24 +3673,24 @@
     </row>
     <row r="57" spans="1:25">
       <c r="A57" s="33"/>
-      <c r="E57" s="45" t="s">
-        <v>1</v>
-      </c>
-      <c r="F57" s="46"/>
-      <c r="G57" s="46"/>
-      <c r="H57" s="46"/>
-      <c r="I57" s="47"/>
-      <c r="J57" s="57"/>
-      <c r="K57" s="58"/>
-      <c r="L57" s="58"/>
-      <c r="M57" s="58"/>
-      <c r="N57" s="58"/>
-      <c r="O57" s="58"/>
-      <c r="P57" s="58"/>
-      <c r="Q57" s="58"/>
-      <c r="R57" s="58"/>
-      <c r="S57" s="58"/>
-      <c r="T57" s="59"/>
+      <c r="E57" s="37" t="s">
+        <v>1</v>
+      </c>
+      <c r="F57" s="38"/>
+      <c r="G57" s="38"/>
+      <c r="H57" s="38"/>
+      <c r="I57" s="39"/>
+      <c r="J57" s="49"/>
+      <c r="K57" s="50"/>
+      <c r="L57" s="50"/>
+      <c r="M57" s="50"/>
+      <c r="N57" s="50"/>
+      <c r="O57" s="50"/>
+      <c r="P57" s="50"/>
+      <c r="Q57" s="50"/>
+      <c r="R57" s="50"/>
+      <c r="S57" s="50"/>
+      <c r="T57" s="51"/>
     </row>
     <row r="58" spans="1:25">
       <c r="A58" s="33" t="s">
@@ -3717,28 +3763,28 @@
     </row>
     <row r="60" spans="1:25">
       <c r="A60" s="33"/>
-      <c r="E60" s="45" t="s">
-        <v>1</v>
-      </c>
-      <c r="F60" s="46"/>
-      <c r="G60" s="46"/>
-      <c r="H60" s="46"/>
-      <c r="I60" s="47"/>
-      <c r="J60" s="57"/>
-      <c r="K60" s="58"/>
-      <c r="L60" s="59"/>
-      <c r="M60" s="51" t="s">
+      <c r="E60" s="37" t="s">
+        <v>1</v>
+      </c>
+      <c r="F60" s="38"/>
+      <c r="G60" s="38"/>
+      <c r="H60" s="38"/>
+      <c r="I60" s="39"/>
+      <c r="J60" s="49"/>
+      <c r="K60" s="50"/>
+      <c r="L60" s="51"/>
+      <c r="M60" s="43" t="s">
         <v>48</v>
       </c>
-      <c r="N60" s="52"/>
-      <c r="O60" s="52"/>
-      <c r="P60" s="53"/>
-      <c r="Q60" s="54" t="s">
+      <c r="N60" s="44"/>
+      <c r="O60" s="44"/>
+      <c r="P60" s="45"/>
+      <c r="Q60" s="46" t="s">
         <v>49</v>
       </c>
-      <c r="R60" s="55"/>
-      <c r="S60" s="55"/>
-      <c r="T60" s="56"/>
+      <c r="R60" s="47"/>
+      <c r="S60" s="47"/>
+      <c r="T60" s="48"/>
     </row>
     <row r="61" spans="1:25">
       <c r="A61" s="33" t="s">
@@ -3811,28 +3857,28 @@
     </row>
     <row r="63" spans="1:25">
       <c r="A63" s="33"/>
-      <c r="E63" s="45" t="s">
-        <v>1</v>
-      </c>
-      <c r="F63" s="46"/>
-      <c r="G63" s="46"/>
-      <c r="H63" s="46"/>
-      <c r="I63" s="47"/>
-      <c r="J63" s="57"/>
-      <c r="K63" s="58"/>
-      <c r="L63" s="59"/>
-      <c r="M63" s="51" t="s">
+      <c r="E63" s="37" t="s">
+        <v>1</v>
+      </c>
+      <c r="F63" s="38"/>
+      <c r="G63" s="38"/>
+      <c r="H63" s="38"/>
+      <c r="I63" s="39"/>
+      <c r="J63" s="49"/>
+      <c r="K63" s="50"/>
+      <c r="L63" s="51"/>
+      <c r="M63" s="43" t="s">
         <v>48</v>
       </c>
-      <c r="N63" s="52"/>
-      <c r="O63" s="52"/>
-      <c r="P63" s="53"/>
-      <c r="Q63" s="54" t="s">
+      <c r="N63" s="44"/>
+      <c r="O63" s="44"/>
+      <c r="P63" s="45"/>
+      <c r="Q63" s="46" t="s">
         <v>49</v>
       </c>
-      <c r="R63" s="55"/>
-      <c r="S63" s="55"/>
-      <c r="T63" s="56"/>
+      <c r="R63" s="47"/>
+      <c r="S63" s="47"/>
+      <c r="T63" s="48"/>
     </row>
     <row r="64" spans="1:25">
       <c r="A64" s="33" t="s">
@@ -3904,30 +3950,30 @@
       <c r="A65" s="33"/>
     </row>
     <row r="66" spans="1:25">
-      <c r="E66" s="45" t="s">
-        <v>1</v>
-      </c>
-      <c r="F66" s="46"/>
-      <c r="G66" s="46"/>
-      <c r="H66" s="46"/>
-      <c r="I66" s="47"/>
-      <c r="J66" s="48" t="s">
+      <c r="E66" s="37" t="s">
+        <v>1</v>
+      </c>
+      <c r="F66" s="38"/>
+      <c r="G66" s="38"/>
+      <c r="H66" s="38"/>
+      <c r="I66" s="39"/>
+      <c r="J66" s="40" t="s">
         <v>47</v>
       </c>
-      <c r="K66" s="49"/>
-      <c r="L66" s="50"/>
-      <c r="M66" s="51" t="s">
+      <c r="K66" s="41"/>
+      <c r="L66" s="42"/>
+      <c r="M66" s="43" t="s">
         <v>48</v>
       </c>
-      <c r="N66" s="52"/>
-      <c r="O66" s="52"/>
-      <c r="P66" s="53"/>
-      <c r="Q66" s="54" t="s">
+      <c r="N66" s="44"/>
+      <c r="O66" s="44"/>
+      <c r="P66" s="45"/>
+      <c r="Q66" s="46" t="s">
         <v>49</v>
       </c>
-      <c r="R66" s="55"/>
-      <c r="S66" s="55"/>
-      <c r="T66" s="56"/>
+      <c r="R66" s="47"/>
+      <c r="S66" s="47"/>
+      <c r="T66" s="48"/>
     </row>
     <row r="67" spans="1:25">
       <c r="A67" s="33" t="s">
@@ -3997,6 +4043,61 @@
     </row>
   </sheetData>
   <mergeCells count="67">
+    <mergeCell ref="E3:I3"/>
+    <mergeCell ref="K3:O3"/>
+    <mergeCell ref="P3:T3"/>
+    <mergeCell ref="E17:I17"/>
+    <mergeCell ref="J17:L17"/>
+    <mergeCell ref="M17:P17"/>
+    <mergeCell ref="Q17:T17"/>
+    <mergeCell ref="E24:I24"/>
+    <mergeCell ref="J24:L24"/>
+    <mergeCell ref="M24:P24"/>
+    <mergeCell ref="Q24:T24"/>
+    <mergeCell ref="E27:I27"/>
+    <mergeCell ref="J27:L27"/>
+    <mergeCell ref="M27:P27"/>
+    <mergeCell ref="Q27:T27"/>
+    <mergeCell ref="E30:I30"/>
+    <mergeCell ref="J30:L30"/>
+    <mergeCell ref="M30:P30"/>
+    <mergeCell ref="Q30:T30"/>
+    <mergeCell ref="E33:I33"/>
+    <mergeCell ref="J33:L33"/>
+    <mergeCell ref="M33:P33"/>
+    <mergeCell ref="Q33:T33"/>
+    <mergeCell ref="E36:I36"/>
+    <mergeCell ref="J36:L36"/>
+    <mergeCell ref="M36:P36"/>
+    <mergeCell ref="Q36:T36"/>
+    <mergeCell ref="E39:I39"/>
+    <mergeCell ref="J39:L39"/>
+    <mergeCell ref="M39:P39"/>
+    <mergeCell ref="Q39:T39"/>
+    <mergeCell ref="E42:I42"/>
+    <mergeCell ref="J42:L42"/>
+    <mergeCell ref="M42:P42"/>
+    <mergeCell ref="Q42:T42"/>
+    <mergeCell ref="E45:I45"/>
+    <mergeCell ref="J45:L45"/>
+    <mergeCell ref="M45:P45"/>
+    <mergeCell ref="Q45:T45"/>
+    <mergeCell ref="E48:I48"/>
+    <mergeCell ref="J48:L48"/>
+    <mergeCell ref="M48:P48"/>
+    <mergeCell ref="Q48:T48"/>
+    <mergeCell ref="E51:I51"/>
+    <mergeCell ref="J51:L51"/>
+    <mergeCell ref="M51:P51"/>
+    <mergeCell ref="Q51:T51"/>
+    <mergeCell ref="E54:I54"/>
+    <mergeCell ref="J54:L54"/>
+    <mergeCell ref="M54:P54"/>
+    <mergeCell ref="Q54:T54"/>
+    <mergeCell ref="E57:I57"/>
+    <mergeCell ref="J57:L57"/>
+    <mergeCell ref="M57:P57"/>
+    <mergeCell ref="Q57:T57"/>
     <mergeCell ref="E66:I66"/>
     <mergeCell ref="J66:L66"/>
     <mergeCell ref="M66:P66"/>
@@ -4009,61 +4110,6 @@
     <mergeCell ref="J63:L63"/>
     <mergeCell ref="M63:P63"/>
     <mergeCell ref="Q63:T63"/>
-    <mergeCell ref="E54:I54"/>
-    <mergeCell ref="J54:L54"/>
-    <mergeCell ref="M54:P54"/>
-    <mergeCell ref="Q54:T54"/>
-    <mergeCell ref="E57:I57"/>
-    <mergeCell ref="J57:L57"/>
-    <mergeCell ref="M57:P57"/>
-    <mergeCell ref="Q57:T57"/>
-    <mergeCell ref="E48:I48"/>
-    <mergeCell ref="J48:L48"/>
-    <mergeCell ref="M48:P48"/>
-    <mergeCell ref="Q48:T48"/>
-    <mergeCell ref="E51:I51"/>
-    <mergeCell ref="J51:L51"/>
-    <mergeCell ref="M51:P51"/>
-    <mergeCell ref="Q51:T51"/>
-    <mergeCell ref="E42:I42"/>
-    <mergeCell ref="J42:L42"/>
-    <mergeCell ref="M42:P42"/>
-    <mergeCell ref="Q42:T42"/>
-    <mergeCell ref="E45:I45"/>
-    <mergeCell ref="J45:L45"/>
-    <mergeCell ref="M45:P45"/>
-    <mergeCell ref="Q45:T45"/>
-    <mergeCell ref="E36:I36"/>
-    <mergeCell ref="J36:L36"/>
-    <mergeCell ref="M36:P36"/>
-    <mergeCell ref="Q36:T36"/>
-    <mergeCell ref="E39:I39"/>
-    <mergeCell ref="J39:L39"/>
-    <mergeCell ref="M39:P39"/>
-    <mergeCell ref="Q39:T39"/>
-    <mergeCell ref="E30:I30"/>
-    <mergeCell ref="J30:L30"/>
-    <mergeCell ref="M30:P30"/>
-    <mergeCell ref="Q30:T30"/>
-    <mergeCell ref="E33:I33"/>
-    <mergeCell ref="J33:L33"/>
-    <mergeCell ref="M33:P33"/>
-    <mergeCell ref="Q33:T33"/>
-    <mergeCell ref="E24:I24"/>
-    <mergeCell ref="J24:L24"/>
-    <mergeCell ref="M24:P24"/>
-    <mergeCell ref="Q24:T24"/>
-    <mergeCell ref="E27:I27"/>
-    <mergeCell ref="J27:L27"/>
-    <mergeCell ref="M27:P27"/>
-    <mergeCell ref="Q27:T27"/>
-    <mergeCell ref="E3:I3"/>
-    <mergeCell ref="K3:O3"/>
-    <mergeCell ref="P3:T3"/>
-    <mergeCell ref="E17:I17"/>
-    <mergeCell ref="J17:L17"/>
-    <mergeCell ref="M17:P17"/>
-    <mergeCell ref="Q17:T17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
@@ -4072,7 +4118,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A52"/>
+  <dimension ref="A1:A54"/>
   <sheetFormatPr defaultRowHeight="14.6"/>
   <cols>
     <col min="1" max="1" width="96.765625" customWidth="1"/>
@@ -4298,7 +4344,18 @@
         <v>144</v>
       </c>
     </row>
+    <row r="53" spans="1:1">
+      <c r="A53" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1">
+      <c r="A54" t="s">
+        <v>146</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>